<commit_message>
Use core product-line GMV as base and add per-line breakdown
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KG85ckxG9s6f8ED7eTkqJz
</commit_message>
<xml_diff>
--- a/output/KOL岗位产值测算.xlsx
+++ b/output/KOL岗位产值测算.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="参数" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="月度测算" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="品线拆分" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -119,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="98">
   <si>
     <r>
       <rPr>
@@ -348,7 +349,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">示例值，请替换为实际负责账号的月均销售额（多个账号填合计）。也可在「月度测算」第</t>
+      <t xml:space="preserve">取下方</t>
     </r>
     <r>
       <rPr>
@@ -365,6 +366,40 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">个核心品线月均</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合计（美国站，用户提供）。也可在「月度测算」第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">行逐月覆盖以体现淡旺季。</t>
     </r>
   </si>
@@ -1077,6 +1112,139 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">核心品线（美国站）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月均</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">占比</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（可增删品线，保持在第</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19–24</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行内）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">油泵</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用户提供：美国站月均</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">充气泵</t>
+  </si>
+  <si>
+    <t xml:space="preserve">逆变器</t>
+  </si>
+  <si>
+    <t xml:space="preserve">冲击扳手</t>
+  </si>
+  <si>
+    <t xml:space="preserve">黄油枪</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工作灯</t>
+  </si>
+  <si>
+    <t xml:space="preserve">合计</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -2102,6 +2270,386 @@
   </si>
   <si>
     <t xml:space="preserve">跑通之后的长期门槛，低于这个体量建议一人覆盖多个账号。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">全年增量按品线拆分（按</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">占比分摊，各品线占比口径相同）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">如某品线达人资源更好</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">更差，可后续改为分品线占比；当前为平均口径。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">品线</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">全年</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">现有</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ACC</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">基线（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ACC</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">放量增量（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">社媒</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KOL</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新增（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">岗位增量合计（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">增量毛利（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">增量占</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GMV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">校验：岗位增量合计应等于「月度测算」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">N13 →</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2115,7 +2663,7 @@
     <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="168" formatCode="0.0\x"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2193,22 +2741,15 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF008000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2218,6 +2759,13 @@
       <sz val="11"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2240,6 +2788,12 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -2324,7 +2878,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2345,7 +2899,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2353,15 +2907,35 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2381,11 +2955,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2393,7 +2963,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2401,15 +2971,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2417,7 +2979,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2425,11 +2987,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2438,6 +2996,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2693,7 +3263,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2729,7 +3299,8 @@
         <v>5</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>300000</v>
+        <f aca="false">SUM(B19:B24)</f>
+        <v>1380000</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>6</v>
@@ -2783,7 +3354,7 @@
       <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="10" t="n">
         <v>1000</v>
       </c>
       <c r="E10" s="6" t="s">
@@ -2794,7 +3365,7 @@
       <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="10" t="n">
         <v>2000</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -2850,6 +3421,129 @@
       </c>
       <c r="E15" s="6" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <f aca="false">IFERROR(B19/$B$25,0)</f>
+        <v>0.144927536231884</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <f aca="false">IFERROR(B20/$B$25,0)</f>
+        <v>0.181159420289855</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>340000</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <f aca="false">IFERROR(B21/$B$25,0)</f>
+        <v>0.246376811594203</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>260000</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <f aca="false">IFERROR(B22/$B$25,0)</f>
+        <v>0.188405797101449</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>130000</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <f aca="false">IFERROR(B23/$B$25,0)</f>
+        <v>0.0942028985507246</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <f aca="false">IFERROR(B24/$B$25,0)</f>
+        <v>0.144927536231884</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="13" t="n">
+        <f aca="false">SUM(B19:B24)</f>
+        <v>1380000</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <f aca="false">SUM(C19:C24)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2876,1290 +3570,1290 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>27</v>
+      <c r="A1" s="15" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K4" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="M4" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="B4" s="16" t="s">
         <v>42</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="13"/>
+        <v>55</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="N5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="C6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="C6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="D6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="D6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="E6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="E6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="F6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="F6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="G6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="G6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="H6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="H6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="I6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="I6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="J6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="J6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="K6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="K6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="L6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="L6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="M6" s="14" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="M6" s="19" t="n">
         <f aca="false">参数!$B$5</f>
-        <v>300000</v>
-      </c>
-      <c r="N6" s="15" t="n">
+        <v>1380000</v>
+      </c>
+      <c r="N6" s="13" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>3600000</v>
+        <v>16560000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="B7" s="20" t="n">
         <f aca="false">B6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="C7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="C7" s="20" t="n">
         <f aca="false">C6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="D7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="D7" s="20" t="n">
         <f aca="false">D6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="E7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="E7" s="20" t="n">
         <f aca="false">E6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="F7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="F7" s="20" t="n">
         <f aca="false">F6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="G7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="G7" s="20" t="n">
         <f aca="false">G6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="H7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="H7" s="20" t="n">
         <f aca="false">H6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="I7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="I7" s="20" t="n">
         <f aca="false">I6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="J7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="J7" s="20" t="n">
         <f aca="false">J6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="K7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="K7" s="20" t="n">
         <f aca="false">K6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="L7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="L7" s="20" t="n">
         <f aca="false">L6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="M7" s="16" t="n">
+        <v>72450</v>
+      </c>
+      <c r="M7" s="20" t="n">
         <f aca="false">M6*参数!$B$6</f>
-        <v>15750</v>
-      </c>
-      <c r="N7" s="15" t="n">
+        <v>72450</v>
+      </c>
+      <c r="N7" s="13" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>189000</v>
+        <v>869400</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
+      <c r="A8" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="19" t="n">
+        <v>61</v>
+      </c>
+      <c r="B9" s="23" t="n">
         <f aca="false">IF(1&lt;=3,参数!$B$14,IF(1&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.005</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">IF(2&lt;=3,参数!$B$14,IF(2&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.005</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="23" t="n">
         <f aca="false">IF(3&lt;=3,参数!$B$14,IF(3&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.005</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="23" t="n">
         <f aca="false">IF(4&lt;=3,参数!$B$14,IF(4&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.01</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="23" t="n">
         <f aca="false">IF(5&lt;=3,参数!$B$14,IF(5&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.01</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="23" t="n">
         <f aca="false">IF(6&lt;=3,参数!$B$14,IF(6&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.01</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="23" t="n">
         <f aca="false">IF(7&lt;=3,参数!$B$14,IF(7&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="23" t="n">
         <f aca="false">IF(8&lt;=3,参数!$B$14,IF(8&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="23" t="n">
         <f aca="false">IF(9&lt;=3,参数!$B$14,IF(9&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="23" t="n">
         <f aca="false">IF(10&lt;=3,参数!$B$14,IF(10&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="L9" s="23" t="n">
         <f aca="false">IF(11&lt;=3,参数!$B$14,IF(11&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="M9" s="19" t="n">
+      <c r="M9" s="23" t="n">
         <f aca="false">IF(12&lt;=3,参数!$B$14,IF(12&lt;=6,参数!$C$14,参数!$D$14))</f>
         <v>0.015</v>
       </c>
-      <c r="N9" s="20" t="n">
+      <c r="N9" s="14" t="n">
         <f aca="false">IFERROR(N10/N6,0)</f>
         <v>0.01125</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="16" t="n">
+        <v>62</v>
+      </c>
+      <c r="B10" s="20" t="n">
         <f aca="false">B6*B9</f>
-        <v>1500</v>
-      </c>
-      <c r="C10" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="C10" s="20" t="n">
         <f aca="false">C6*C9</f>
-        <v>1500</v>
-      </c>
-      <c r="D10" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D10" s="20" t="n">
         <f aca="false">D6*D9</f>
-        <v>1500</v>
-      </c>
-      <c r="E10" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <f aca="false">E6*E9</f>
-        <v>3000</v>
-      </c>
-      <c r="F10" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="F10" s="20" t="n">
         <f aca="false">F6*F9</f>
-        <v>3000</v>
-      </c>
-      <c r="G10" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="G10" s="20" t="n">
         <f aca="false">G6*G9</f>
-        <v>3000</v>
-      </c>
-      <c r="H10" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="H10" s="20" t="n">
         <f aca="false">H6*H9</f>
-        <v>4500</v>
-      </c>
-      <c r="I10" s="16" t="n">
+        <v>20700</v>
+      </c>
+      <c r="I10" s="20" t="n">
         <f aca="false">I6*I9</f>
-        <v>4500</v>
-      </c>
-      <c r="J10" s="16" t="n">
+        <v>20700</v>
+      </c>
+      <c r="J10" s="20" t="n">
         <f aca="false">J6*J9</f>
-        <v>4500</v>
-      </c>
-      <c r="K10" s="16" t="n">
+        <v>20700</v>
+      </c>
+      <c r="K10" s="20" t="n">
         <f aca="false">K6*K9</f>
-        <v>4500</v>
-      </c>
-      <c r="L10" s="16" t="n">
+        <v>20700</v>
+      </c>
+      <c r="L10" s="20" t="n">
         <f aca="false">L6*L9</f>
-        <v>4500</v>
-      </c>
-      <c r="M10" s="16" t="n">
+        <v>20700</v>
+      </c>
+      <c r="M10" s="20" t="n">
         <f aca="false">M6*M9</f>
-        <v>4500</v>
-      </c>
-      <c r="N10" s="15" t="n">
+        <v>20700</v>
+      </c>
+      <c r="N10" s="13" t="n">
         <f aca="false">SUM(B10:M10)</f>
-        <v>40500</v>
+        <v>186300</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="23" t="n">
         <f aca="false">IF(1&lt;=3,参数!$B$15,IF(1&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">IF(2&lt;=3,参数!$B$15,IF(2&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="23" t="n">
         <f aca="false">IF(3&lt;=3,参数!$B$15,IF(3&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="23" t="n">
         <f aca="false">IF(4&lt;=3,参数!$B$15,IF(4&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.01</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="23" t="n">
         <f aca="false">IF(5&lt;=3,参数!$B$15,IF(5&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.01</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="23" t="n">
         <f aca="false">IF(6&lt;=3,参数!$B$15,IF(6&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.01</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="23" t="n">
         <f aca="false">IF(7&lt;=3,参数!$B$15,IF(7&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="23" t="n">
         <f aca="false">IF(8&lt;=3,参数!$B$15,IF(8&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="23" t="n">
         <f aca="false">IF(9&lt;=3,参数!$B$15,IF(9&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="23" t="n">
         <f aca="false">IF(10&lt;=3,参数!$B$15,IF(10&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="L11" s="19" t="n">
+      <c r="L11" s="23" t="n">
         <f aca="false">IF(11&lt;=3,参数!$B$15,IF(11&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="M11" s="19" t="n">
+      <c r="M11" s="23" t="n">
         <f aca="false">IF(12&lt;=3,参数!$B$15,IF(12&lt;=6,参数!$C$15,参数!$D$15))</f>
         <v>0.02</v>
       </c>
-      <c r="N11" s="20" t="n">
+      <c r="N11" s="14" t="n">
         <f aca="false">IFERROR(N12/N6,0)</f>
         <v>0.0125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" s="16" t="n">
+        <v>63</v>
+      </c>
+      <c r="B12" s="20" t="n">
         <f aca="false">B6*B11</f>
         <v>0</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="20" t="n">
         <f aca="false">C6*C11</f>
         <v>0</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="20" t="n">
         <f aca="false">D6*D11</f>
         <v>0</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="20" t="n">
         <f aca="false">E6*E11</f>
-        <v>3000</v>
-      </c>
-      <c r="F12" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="F12" s="20" t="n">
         <f aca="false">F6*F11</f>
-        <v>3000</v>
-      </c>
-      <c r="G12" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="G12" s="20" t="n">
         <f aca="false">G6*G11</f>
-        <v>3000</v>
-      </c>
-      <c r="H12" s="16" t="n">
+        <v>13800</v>
+      </c>
+      <c r="H12" s="20" t="n">
         <f aca="false">H6*H11</f>
-        <v>6000</v>
-      </c>
-      <c r="I12" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="I12" s="20" t="n">
         <f aca="false">I6*I11</f>
-        <v>6000</v>
-      </c>
-      <c r="J12" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="J12" s="20" t="n">
         <f aca="false">J6*J11</f>
-        <v>6000</v>
-      </c>
-      <c r="K12" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="K12" s="20" t="n">
         <f aca="false">K6*K11</f>
-        <v>6000</v>
-      </c>
-      <c r="L12" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="L12" s="20" t="n">
         <f aca="false">L6*L11</f>
-        <v>6000</v>
-      </c>
-      <c r="M12" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="M12" s="20" t="n">
         <f aca="false">M6*M11</f>
-        <v>6000</v>
-      </c>
-      <c r="N12" s="15" t="n">
+        <v>27600</v>
+      </c>
+      <c r="N12" s="13" t="n">
         <f aca="false">SUM(B12:M12)</f>
-        <v>45000</v>
+        <v>207000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="16" t="n">
+      <c r="A13" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="20" t="n">
         <f aca="false">B10+B12</f>
-        <v>1500</v>
-      </c>
-      <c r="C13" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="C13" s="20" t="n">
         <f aca="false">C10+C12</f>
-        <v>1500</v>
-      </c>
-      <c r="D13" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D13" s="20" t="n">
         <f aca="false">D10+D12</f>
-        <v>1500</v>
-      </c>
-      <c r="E13" s="16" t="n">
+        <v>6900</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <f aca="false">E10+E12</f>
-        <v>6000</v>
-      </c>
-      <c r="F13" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="F13" s="20" t="n">
         <f aca="false">F10+F12</f>
-        <v>6000</v>
-      </c>
-      <c r="G13" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="G13" s="20" t="n">
         <f aca="false">G10+G12</f>
-        <v>6000</v>
-      </c>
-      <c r="H13" s="16" t="n">
+        <v>27600</v>
+      </c>
+      <c r="H13" s="20" t="n">
         <f aca="false">H10+H12</f>
-        <v>10500</v>
-      </c>
-      <c r="I13" s="16" t="n">
+        <v>48300</v>
+      </c>
+      <c r="I13" s="20" t="n">
         <f aca="false">I10+I12</f>
-        <v>10500</v>
-      </c>
-      <c r="J13" s="16" t="n">
+        <v>48300</v>
+      </c>
+      <c r="J13" s="20" t="n">
         <f aca="false">J10+J12</f>
-        <v>10500</v>
-      </c>
-      <c r="K13" s="16" t="n">
+        <v>48300</v>
+      </c>
+      <c r="K13" s="20" t="n">
         <f aca="false">K10+K12</f>
-        <v>10500</v>
-      </c>
-      <c r="L13" s="16" t="n">
+        <v>48300</v>
+      </c>
+      <c r="L13" s="20" t="n">
         <f aca="false">L10+L12</f>
-        <v>10500</v>
-      </c>
-      <c r="M13" s="16" t="n">
+        <v>48300</v>
+      </c>
+      <c r="M13" s="20" t="n">
         <f aca="false">M10+M12</f>
-        <v>10500</v>
-      </c>
-      <c r="N13" s="15" t="n">
+        <v>48300</v>
+      </c>
+      <c r="N13" s="13" t="n">
         <f aca="false">SUM(B13:M13)</f>
-        <v>85500</v>
+        <v>393300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="22" t="n">
+        <v>65</v>
+      </c>
+      <c r="B14" s="24" t="n">
         <f aca="false">IFERROR(B13/B6,0)</f>
         <v>0.005</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <f aca="false">IFERROR(C13/C6,0)</f>
         <v>0.005</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="24" t="n">
         <f aca="false">IFERROR(D13/D6,0)</f>
         <v>0.005</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="24" t="n">
         <f aca="false">IFERROR(E13/E6,0)</f>
         <v>0.02</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="24" t="n">
         <f aca="false">IFERROR(F13/F6,0)</f>
         <v>0.02</v>
       </c>
-      <c r="G14" s="22" t="n">
+      <c r="G14" s="24" t="n">
         <f aca="false">IFERROR(G13/G6,0)</f>
         <v>0.02</v>
       </c>
-      <c r="H14" s="22" t="n">
+      <c r="H14" s="24" t="n">
         <f aca="false">IFERROR(H13/H6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="I14" s="24" t="n">
         <f aca="false">IFERROR(I13/I6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="J14" s="24" t="n">
         <f aca="false">IFERROR(J13/J6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="K14" s="22" t="n">
+      <c r="K14" s="24" t="n">
         <f aca="false">IFERROR(K13/K6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="L14" s="22" t="n">
+      <c r="L14" s="24" t="n">
         <f aca="false">IFERROR(L13/L6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="M14" s="22" t="n">
+      <c r="M14" s="24" t="n">
         <f aca="false">IFERROR(M13/M6,0)</f>
         <v>0.035</v>
       </c>
-      <c r="N14" s="23" t="n">
+      <c r="N14" s="25" t="n">
         <f aca="false">IFERROR(N13/N6,0)</f>
         <v>0.02375</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="22" t="n">
+        <v>66</v>
+      </c>
+      <c r="B15" s="24" t="n">
         <f aca="false">参数!$B$6+B9</f>
         <v>0.0575</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="24" t="n">
         <f aca="false">参数!$B$6+C9</f>
         <v>0.0575</v>
       </c>
-      <c r="D15" s="22" t="n">
+      <c r="D15" s="24" t="n">
         <f aca="false">参数!$B$6+D9</f>
         <v>0.0575</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="24" t="n">
         <f aca="false">参数!$B$6+E9</f>
         <v>0.0625</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="24" t="n">
         <f aca="false">参数!$B$6+F9</f>
         <v>0.0625</v>
       </c>
-      <c r="G15" s="22" t="n">
+      <c r="G15" s="24" t="n">
         <f aca="false">参数!$B$6+G9</f>
         <v>0.0625</v>
       </c>
-      <c r="H15" s="22" t="n">
+      <c r="H15" s="24" t="n">
         <f aca="false">参数!$B$6+H9</f>
         <v>0.0675</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="I15" s="24" t="n">
         <f aca="false">参数!$B$6+I9</f>
         <v>0.0675</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="J15" s="24" t="n">
         <f aca="false">参数!$B$6+J9</f>
         <v>0.0675</v>
       </c>
-      <c r="K15" s="22" t="n">
+      <c r="K15" s="24" t="n">
         <f aca="false">参数!$B$6+K9</f>
         <v>0.0675</v>
       </c>
-      <c r="L15" s="22" t="n">
+      <c r="L15" s="24" t="n">
         <f aca="false">参数!$B$6+L9</f>
         <v>0.0675</v>
       </c>
-      <c r="M15" s="22" t="n">
+      <c r="M15" s="24" t="n">
         <f aca="false">参数!$B$6+M9</f>
         <v>0.0675</v>
       </c>
-      <c r="N15" s="23" t="n">
+      <c r="N15" s="25" t="n">
         <f aca="false">IFERROR((N7+N10)/N6,0)</f>
         <v>0.06375</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
+      <c r="A17" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="16" t="n">
+        <v>68</v>
+      </c>
+      <c r="B18" s="20" t="n">
         <f aca="false">B13*参数!$B$7</f>
-        <v>450</v>
-      </c>
-      <c r="C18" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="C18" s="20" t="n">
         <f aca="false">C13*参数!$B$7</f>
-        <v>450</v>
-      </c>
-      <c r="D18" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="D18" s="20" t="n">
         <f aca="false">D13*参数!$B$7</f>
-        <v>450</v>
-      </c>
-      <c r="E18" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="E18" s="20" t="n">
         <f aca="false">E13*参数!$B$7</f>
-        <v>1800</v>
-      </c>
-      <c r="F18" s="16" t="n">
+        <v>8280</v>
+      </c>
+      <c r="F18" s="20" t="n">
         <f aca="false">F13*参数!$B$7</f>
-        <v>1800</v>
-      </c>
-      <c r="G18" s="16" t="n">
+        <v>8280</v>
+      </c>
+      <c r="G18" s="20" t="n">
         <f aca="false">G13*参数!$B$7</f>
-        <v>1800</v>
-      </c>
-      <c r="H18" s="16" t="n">
+        <v>8280</v>
+      </c>
+      <c r="H18" s="20" t="n">
         <f aca="false">H13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="I18" s="16" t="n">
+        <v>14490</v>
+      </c>
+      <c r="I18" s="20" t="n">
         <f aca="false">I13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="J18" s="16" t="n">
+        <v>14490</v>
+      </c>
+      <c r="J18" s="20" t="n">
         <f aca="false">J13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="K18" s="16" t="n">
+        <v>14490</v>
+      </c>
+      <c r="K18" s="20" t="n">
         <f aca="false">K13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="L18" s="16" t="n">
+        <v>14490</v>
+      </c>
+      <c r="L18" s="20" t="n">
         <f aca="false">L13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="M18" s="16" t="n">
+        <v>14490</v>
+      </c>
+      <c r="M18" s="20" t="n">
         <f aca="false">M13*参数!$B$7</f>
-        <v>3150</v>
-      </c>
-      <c r="N18" s="15" t="n">
+        <v>14490</v>
+      </c>
+      <c r="N18" s="13" t="n">
         <f aca="false">SUM(B18:M18)</f>
-        <v>25650</v>
+        <v>117990</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="16" t="n">
+        <v>69</v>
+      </c>
+      <c r="B19" s="20" t="n">
         <f aca="false">B10*参数!$B$8</f>
-        <v>150</v>
-      </c>
-      <c r="C19" s="16" t="n">
+        <v>690</v>
+      </c>
+      <c r="C19" s="20" t="n">
         <f aca="false">C10*参数!$B$8</f>
-        <v>150</v>
-      </c>
-      <c r="D19" s="16" t="n">
+        <v>690</v>
+      </c>
+      <c r="D19" s="20" t="n">
         <f aca="false">D10*参数!$B$8</f>
-        <v>150</v>
-      </c>
-      <c r="E19" s="16" t="n">
+        <v>690</v>
+      </c>
+      <c r="E19" s="20" t="n">
         <f aca="false">E10*参数!$B$8</f>
-        <v>300</v>
-      </c>
-      <c r="F19" s="16" t="n">
+        <v>1380</v>
+      </c>
+      <c r="F19" s="20" t="n">
         <f aca="false">F10*参数!$B$8</f>
-        <v>300</v>
-      </c>
-      <c r="G19" s="16" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G19" s="20" t="n">
         <f aca="false">G10*参数!$B$8</f>
-        <v>300</v>
-      </c>
-      <c r="H19" s="16" t="n">
+        <v>1380</v>
+      </c>
+      <c r="H19" s="20" t="n">
         <f aca="false">H10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="I19" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="I19" s="20" t="n">
         <f aca="false">I10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="J19" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="J19" s="20" t="n">
         <f aca="false">J10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="K19" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="K19" s="20" t="n">
         <f aca="false">K10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="L19" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="L19" s="20" t="n">
         <f aca="false">L10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="M19" s="16" t="n">
+        <v>2070</v>
+      </c>
+      <c r="M19" s="20" t="n">
         <f aca="false">M10*参数!$B$8</f>
-        <v>450</v>
-      </c>
-      <c r="N19" s="15" t="n">
+        <v>2070</v>
+      </c>
+      <c r="N19" s="13" t="n">
         <f aca="false">SUM(B19:M19)</f>
-        <v>4050</v>
+        <v>18630</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="B20" s="20" t="n">
         <f aca="false">B12*参数!$B$9</f>
         <v>0</v>
       </c>
-      <c r="C20" s="16" t="n">
+      <c r="C20" s="20" t="n">
         <f aca="false">C12*参数!$B$9</f>
         <v>0</v>
       </c>
-      <c r="D20" s="16" t="n">
+      <c r="D20" s="20" t="n">
         <f aca="false">D12*参数!$B$9</f>
         <v>0</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E20" s="20" t="n">
         <f aca="false">E12*参数!$B$9</f>
-        <v>600</v>
-      </c>
-      <c r="F20" s="16" t="n">
+        <v>2760</v>
+      </c>
+      <c r="F20" s="20" t="n">
         <f aca="false">F12*参数!$B$9</f>
-        <v>600</v>
-      </c>
-      <c r="G20" s="16" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G20" s="20" t="n">
         <f aca="false">G12*参数!$B$9</f>
-        <v>600</v>
-      </c>
-      <c r="H20" s="16" t="n">
+        <v>2760</v>
+      </c>
+      <c r="H20" s="20" t="n">
         <f aca="false">H12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="I20" s="16" t="n">
+        <v>5520</v>
+      </c>
+      <c r="I20" s="20" t="n">
         <f aca="false">I12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="J20" s="16" t="n">
+        <v>5520</v>
+      </c>
+      <c r="J20" s="20" t="n">
         <f aca="false">J12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="K20" s="16" t="n">
+        <v>5520</v>
+      </c>
+      <c r="K20" s="20" t="n">
         <f aca="false">K12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="L20" s="16" t="n">
+        <v>5520</v>
+      </c>
+      <c r="L20" s="20" t="n">
         <f aca="false">L12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="M20" s="16" t="n">
+        <v>5520</v>
+      </c>
+      <c r="M20" s="20" t="n">
         <f aca="false">M12*参数!$B$9</f>
-        <v>1200</v>
-      </c>
-      <c r="N20" s="15" t="n">
+        <v>5520</v>
+      </c>
+      <c r="N20" s="13" t="n">
         <f aca="false">SUM(B20:M20)</f>
-        <v>9000</v>
+        <v>41400</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="16" t="n">
+        <v>71</v>
+      </c>
+      <c r="B21" s="20" t="n">
         <f aca="false">IF(1&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="20" t="n">
         <f aca="false">IF(2&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="D21" s="16" t="n">
+      <c r="D21" s="20" t="n">
         <f aca="false">IF(3&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="E21" s="16" t="n">
+      <c r="E21" s="20" t="n">
         <f aca="false">IF(4&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="F21" s="16" t="n">
+      <c r="F21" s="20" t="n">
         <f aca="false">IF(5&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="G21" s="16" t="n">
+      <c r="G21" s="20" t="n">
         <f aca="false">IF(6&lt;=6,参数!$B$10,0)</f>
         <v>1000</v>
       </c>
-      <c r="H21" s="16" t="n">
+      <c r="H21" s="20" t="n">
         <f aca="false">IF(7&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="I21" s="16" t="n">
+      <c r="I21" s="20" t="n">
         <f aca="false">IF(8&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="16" t="n">
+      <c r="J21" s="20" t="n">
         <f aca="false">IF(9&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="K21" s="16" t="n">
+      <c r="K21" s="20" t="n">
         <f aca="false">IF(10&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="16" t="n">
+      <c r="L21" s="20" t="n">
         <f aca="false">IF(11&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="M21" s="16" t="n">
+      <c r="M21" s="20" t="n">
         <f aca="false">IF(12&lt;=6,参数!$B$10,0)</f>
         <v>0</v>
       </c>
-      <c r="N21" s="15" t="n">
+      <c r="N21" s="13" t="n">
         <f aca="false">SUM(B21:M21)</f>
         <v>6000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" s="14" t="n">
+        <v>72</v>
+      </c>
+      <c r="B22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="F22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="G22" s="14" t="n">
+      <c r="G22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="H22" s="14" t="n">
+      <c r="H22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="I22" s="14" t="n">
+      <c r="I22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="K22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="L22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="M22" s="19" t="n">
         <f aca="false">参数!$B$11</f>
         <v>2000</v>
       </c>
-      <c r="N22" s="15" t="n">
+      <c r="N22" s="13" t="n">
         <f aca="false">SUM(B22:M22)</f>
         <v>24000</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B23" s="16" t="n">
+        <v>73</v>
+      </c>
+      <c r="B23" s="20" t="n">
         <f aca="false">SUM(B19:B22)</f>
-        <v>3150</v>
-      </c>
-      <c r="C23" s="16" t="n">
+        <v>3690</v>
+      </c>
+      <c r="C23" s="20" t="n">
         <f aca="false">SUM(C19:C22)</f>
-        <v>3150</v>
-      </c>
-      <c r="D23" s="16" t="n">
+        <v>3690</v>
+      </c>
+      <c r="D23" s="20" t="n">
         <f aca="false">SUM(D19:D22)</f>
-        <v>3150</v>
-      </c>
-      <c r="E23" s="16" t="n">
+        <v>3690</v>
+      </c>
+      <c r="E23" s="20" t="n">
         <f aca="false">SUM(E19:E22)</f>
-        <v>3900</v>
-      </c>
-      <c r="F23" s="16" t="n">
+        <v>7140</v>
+      </c>
+      <c r="F23" s="20" t="n">
         <f aca="false">SUM(F19:F22)</f>
-        <v>3900</v>
-      </c>
-      <c r="G23" s="16" t="n">
+        <v>7140</v>
+      </c>
+      <c r="G23" s="20" t="n">
         <f aca="false">SUM(G19:G22)</f>
-        <v>3900</v>
-      </c>
-      <c r="H23" s="16" t="n">
+        <v>7140</v>
+      </c>
+      <c r="H23" s="20" t="n">
         <f aca="false">SUM(H19:H22)</f>
-        <v>3650</v>
-      </c>
-      <c r="I23" s="16" t="n">
+        <v>9590</v>
+      </c>
+      <c r="I23" s="20" t="n">
         <f aca="false">SUM(I19:I22)</f>
-        <v>3650</v>
-      </c>
-      <c r="J23" s="16" t="n">
+        <v>9590</v>
+      </c>
+      <c r="J23" s="20" t="n">
         <f aca="false">SUM(J19:J22)</f>
-        <v>3650</v>
-      </c>
-      <c r="K23" s="16" t="n">
+        <v>9590</v>
+      </c>
+      <c r="K23" s="20" t="n">
         <f aca="false">SUM(K19:K22)</f>
-        <v>3650</v>
-      </c>
-      <c r="L23" s="16" t="n">
+        <v>9590</v>
+      </c>
+      <c r="L23" s="20" t="n">
         <f aca="false">SUM(L19:L22)</f>
-        <v>3650</v>
-      </c>
-      <c r="M23" s="16" t="n">
+        <v>9590</v>
+      </c>
+      <c r="M23" s="20" t="n">
         <f aca="false">SUM(M19:M22)</f>
-        <v>3650</v>
-      </c>
-      <c r="N23" s="15" t="n">
+        <v>9590</v>
+      </c>
+      <c r="N23" s="13" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>43050</v>
+        <v>90030</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B24" s="16" t="n">
+      <c r="A24" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="20" t="n">
         <f aca="false">B18-B23</f>
-        <v>-2700</v>
-      </c>
-      <c r="C24" s="16" t="n">
+        <v>-1620</v>
+      </c>
+      <c r="C24" s="20" t="n">
         <f aca="false">C18-C23</f>
-        <v>-2700</v>
-      </c>
-      <c r="D24" s="16" t="n">
+        <v>-1620</v>
+      </c>
+      <c r="D24" s="20" t="n">
         <f aca="false">D18-D23</f>
-        <v>-2700</v>
-      </c>
-      <c r="E24" s="16" t="n">
+        <v>-1620</v>
+      </c>
+      <c r="E24" s="20" t="n">
         <f aca="false">E18-E23</f>
-        <v>-2100</v>
-      </c>
-      <c r="F24" s="16" t="n">
+        <v>1140</v>
+      </c>
+      <c r="F24" s="20" t="n">
         <f aca="false">F18-F23</f>
-        <v>-2100</v>
-      </c>
-      <c r="G24" s="16" t="n">
+        <v>1140</v>
+      </c>
+      <c r="G24" s="20" t="n">
         <f aca="false">G18-G23</f>
-        <v>-2100</v>
-      </c>
-      <c r="H24" s="16" t="n">
+        <v>1140</v>
+      </c>
+      <c r="H24" s="20" t="n">
         <f aca="false">H18-H23</f>
-        <v>-500</v>
-      </c>
-      <c r="I24" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="I24" s="20" t="n">
         <f aca="false">I18-I23</f>
-        <v>-500</v>
-      </c>
-      <c r="J24" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="J24" s="20" t="n">
         <f aca="false">J18-J23</f>
-        <v>-500</v>
-      </c>
-      <c r="K24" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="K24" s="20" t="n">
         <f aca="false">K18-K23</f>
-        <v>-500</v>
-      </c>
-      <c r="L24" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="L24" s="20" t="n">
         <f aca="false">L18-L23</f>
-        <v>-500</v>
-      </c>
-      <c r="M24" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="M24" s="20" t="n">
         <f aca="false">M18-M23</f>
-        <v>-500</v>
-      </c>
-      <c r="N24" s="15" t="n">
+        <v>4900</v>
+      </c>
+      <c r="N24" s="13" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>-17400</v>
+        <v>27960</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" s="16" t="n">
+        <v>75</v>
+      </c>
+      <c r="B25" s="20" t="n">
         <f aca="false">B24</f>
-        <v>-2700</v>
-      </c>
-      <c r="C25" s="16" t="n">
+        <v>-1620</v>
+      </c>
+      <c r="C25" s="20" t="n">
         <f aca="false">B25+C24</f>
-        <v>-5400</v>
-      </c>
-      <c r="D25" s="16" t="n">
+        <v>-3240</v>
+      </c>
+      <c r="D25" s="20" t="n">
         <f aca="false">C25+D24</f>
-        <v>-8100</v>
-      </c>
-      <c r="E25" s="16" t="n">
+        <v>-4860</v>
+      </c>
+      <c r="E25" s="20" t="n">
         <f aca="false">D25+E24</f>
-        <v>-10200</v>
-      </c>
-      <c r="F25" s="16" t="n">
+        <v>-3720</v>
+      </c>
+      <c r="F25" s="20" t="n">
         <f aca="false">E25+F24</f>
-        <v>-12300</v>
-      </c>
-      <c r="G25" s="16" t="n">
+        <v>-2580</v>
+      </c>
+      <c r="G25" s="20" t="n">
         <f aca="false">F25+G24</f>
-        <v>-14400</v>
-      </c>
-      <c r="H25" s="16" t="n">
+        <v>-1440</v>
+      </c>
+      <c r="H25" s="20" t="n">
         <f aca="false">G25+H24</f>
-        <v>-14900</v>
-      </c>
-      <c r="I25" s="16" t="n">
+        <v>3460</v>
+      </c>
+      <c r="I25" s="20" t="n">
         <f aca="false">H25+I24</f>
-        <v>-15400</v>
-      </c>
-      <c r="J25" s="16" t="n">
+        <v>8360</v>
+      </c>
+      <c r="J25" s="20" t="n">
         <f aca="false">I25+J24</f>
-        <v>-15900</v>
-      </c>
-      <c r="K25" s="16" t="n">
+        <v>13260</v>
+      </c>
+      <c r="K25" s="20" t="n">
         <f aca="false">J25+K24</f>
-        <v>-16400</v>
-      </c>
-      <c r="L25" s="16" t="n">
+        <v>18160</v>
+      </c>
+      <c r="L25" s="20" t="n">
         <f aca="false">K25+L24</f>
-        <v>-16900</v>
-      </c>
-      <c r="M25" s="16" t="n">
+        <v>23060</v>
+      </c>
+      <c r="M25" s="20" t="n">
         <f aca="false">L25+M24</f>
-        <v>-17400</v>
-      </c>
-      <c r="N25" s="13"/>
+        <v>27960</v>
+      </c>
+      <c r="N25" s="18"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="24" t="n">
+        <v>76</v>
+      </c>
+      <c r="B26" s="26" t="n">
         <f aca="false">IFERROR(B13/B23,0)</f>
-        <v>0.476190476190476</v>
-      </c>
-      <c r="C26" s="24" t="n">
+        <v>1.86991869918699</v>
+      </c>
+      <c r="C26" s="26" t="n">
         <f aca="false">IFERROR(C13/C23,0)</f>
-        <v>0.476190476190476</v>
-      </c>
-      <c r="D26" s="24" t="n">
+        <v>1.86991869918699</v>
+      </c>
+      <c r="D26" s="26" t="n">
         <f aca="false">IFERROR(D13/D23,0)</f>
-        <v>0.476190476190476</v>
-      </c>
-      <c r="E26" s="24" t="n">
+        <v>1.86991869918699</v>
+      </c>
+      <c r="E26" s="26" t="n">
         <f aca="false">IFERROR(E13/E23,0)</f>
-        <v>1.53846153846154</v>
-      </c>
-      <c r="F26" s="24" t="n">
+        <v>3.8655462184874</v>
+      </c>
+      <c r="F26" s="26" t="n">
         <f aca="false">IFERROR(F13/F23,0)</f>
-        <v>1.53846153846154</v>
-      </c>
-      <c r="G26" s="24" t="n">
+        <v>3.8655462184874</v>
+      </c>
+      <c r="G26" s="26" t="n">
         <f aca="false">IFERROR(G13/G23,0)</f>
-        <v>1.53846153846154</v>
-      </c>
-      <c r="H26" s="24" t="n">
+        <v>3.8655462184874</v>
+      </c>
+      <c r="H26" s="26" t="n">
         <f aca="false">IFERROR(H13/H23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="I26" s="24" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="I26" s="26" t="n">
         <f aca="false">IFERROR(I13/I23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="J26" s="24" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="J26" s="26" t="n">
         <f aca="false">IFERROR(J13/J23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="K26" s="24" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="K26" s="26" t="n">
         <f aca="false">IFERROR(K13/K23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="L26" s="24" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="L26" s="26" t="n">
         <f aca="false">IFERROR(L13/L23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="M26" s="24" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="M26" s="26" t="n">
         <f aca="false">IFERROR(M13/M23,0)</f>
-        <v>2.87671232876712</v>
-      </c>
-      <c r="N26" s="25" t="n">
+        <v>5.03649635036496</v>
+      </c>
+      <c r="N26" s="27" t="n">
         <f aca="false">IFERROR(N13/N23,0)</f>
-        <v>1.98606271777003</v>
+        <v>4.36854381872709</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
+      <c r="A28" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+      <c r="M28" s="22"/>
+      <c r="N28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="26" t="n">
+        <v>78</v>
+      </c>
+      <c r="B29" s="5" t="n">
         <f aca="false">N13</f>
-        <v>85500</v>
-      </c>
-      <c r="C29" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
+        <v>393300</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="28"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B30" s="26" t="n">
+        <v>80</v>
+      </c>
+      <c r="B30" s="5" t="n">
         <f aca="false">N24</f>
-        <v>-17400</v>
-      </c>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
+        <v>27960</v>
+      </c>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="N30" s="28"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31" s="28" t="str">
+        <v>81</v>
+      </c>
+      <c r="B31" s="29" t="str">
         <f aca="false">IFERROR(INDEX($B$4:$M$4,MATCH(TRUE(),INDEX($B$24:$M$24&gt;0,0),0)),"12个月内未转正")</f>
-        <v>12个月内未转正</v>
-      </c>
-      <c r="C31" s="27" t="s">
-        <v>70</v>
-      </c>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="27"/>
-      <c r="M31" s="27"/>
-      <c r="N31" s="27"/>
+        <v>第4月</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="28"/>
+      <c r="M31" s="28"/>
+      <c r="N31" s="28"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B32" s="26" t="n">
+        <v>83</v>
+      </c>
+      <c r="B32" s="5" t="n">
         <f aca="false">IFERROR((参数!B11*12+参数!B10*6)/(SUMPRODUCT(B9:M9)*(参数!B7-参数!B8)+SUMPRODUCT(B11:M11)*(参数!B7-参数!B9)),0)</f>
         <v>714285.714285714</v>
       </c>
-      <c r="C32" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="27"/>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="27"/>
-      <c r="M32" s="27"/>
-      <c r="N32" s="27"/>
+      <c r="C32" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="28"/>
+      <c r="L32" s="28"/>
+      <c r="M32" s="28"/>
+      <c r="N32" s="28"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="26" t="n">
+        <v>85</v>
+      </c>
+      <c r="B33" s="5" t="n">
         <f aca="false">IFERROR(参数!B11/(参数!D14*(参数!B7-参数!B8)+参数!D15*(参数!B7-参数!B9)),0)</f>
         <v>400000</v>
       </c>
-      <c r="C33" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
-      <c r="K33" s="27"/>
-      <c r="L33" s="27"/>
-      <c r="M33" s="27"/>
-      <c r="N33" s="27"/>
+      <c r="C33" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="28"/>
+      <c r="L33" s="28"/>
+      <c r="M33" s="28"/>
+      <c r="N33" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4178,4 +4872,316 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="str">
+        <f aca="false">参数!A19</f>
+        <v>油泵</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <f aca="false">参数!B19*12</f>
+        <v>2400000</v>
+      </c>
+      <c r="C5" s="20" t="n">
+        <f aca="false">B5*参数!$B$6</f>
+        <v>126000</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <f aca="false">B5*月度测算!$N$9</f>
+        <v>27000</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <f aca="false">B5*月度测算!$N$11</f>
+        <v>30000</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <f aca="false">D5+E5</f>
+        <v>57000</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <f aca="false">F5*参数!$B$7</f>
+        <v>17100</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <f aca="false">IFERROR(F5/B5,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="str">
+        <f aca="false">参数!A20</f>
+        <v>充气泵</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <f aca="false">参数!B20*12</f>
+        <v>3000000</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <f aca="false">B6*参数!$B$6</f>
+        <v>157500</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <f aca="false">B6*月度测算!$N$9</f>
+        <v>33750</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <f aca="false">B6*月度测算!$N$11</f>
+        <v>37500</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <f aca="false">D6+E6</f>
+        <v>71250</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <f aca="false">F6*参数!$B$7</f>
+        <v>21375</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <f aca="false">IFERROR(F6/B6,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="str">
+        <f aca="false">参数!A21</f>
+        <v>逆变器</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <f aca="false">参数!B21*12</f>
+        <v>4080000</v>
+      </c>
+      <c r="C7" s="20" t="n">
+        <f aca="false">B7*参数!$B$6</f>
+        <v>214200</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">B7*月度测算!$N$9</f>
+        <v>45900</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <f aca="false">B7*月度测算!$N$11</f>
+        <v>51000</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <f aca="false">D7+E7</f>
+        <v>96900</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <f aca="false">F7*参数!$B$7</f>
+        <v>29070</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <f aca="false">IFERROR(F7/B7,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="str">
+        <f aca="false">参数!A22</f>
+        <v>冲击扳手</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <f aca="false">参数!B22*12</f>
+        <v>3120000</v>
+      </c>
+      <c r="C8" s="20" t="n">
+        <f aca="false">B8*参数!$B$6</f>
+        <v>163800</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">B8*月度测算!$N$9</f>
+        <v>35100</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <f aca="false">B8*月度测算!$N$11</f>
+        <v>39000</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <f aca="false">D8+E8</f>
+        <v>74100</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <f aca="false">F8*参数!$B$7</f>
+        <v>22230</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <f aca="false">IFERROR(F8/B8,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="str">
+        <f aca="false">参数!A23</f>
+        <v>黄油枪</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <f aca="false">参数!B23*12</f>
+        <v>1560000</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <f aca="false">B9*参数!$B$6</f>
+        <v>81900</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">B9*月度测算!$N$9</f>
+        <v>17550</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <f aca="false">B9*月度测算!$N$11</f>
+        <v>19500</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <f aca="false">D9+E9</f>
+        <v>37050</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <f aca="false">F9*参数!$B$7</f>
+        <v>11115</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <f aca="false">IFERROR(F9/B9,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="str">
+        <f aca="false">参数!A24</f>
+        <v>工作灯</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <f aca="false">参数!B24*12</f>
+        <v>2400000</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <f aca="false">B10*参数!$B$6</f>
+        <v>126000</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">B10*月度测算!$N$9</f>
+        <v>27000</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <f aca="false">B10*月度测算!$N$11</f>
+        <v>30000</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <f aca="false">D10+E10</f>
+        <v>57000</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <f aca="false">F10*参数!$B$7</f>
+        <v>17100</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <f aca="false">IFERROR(F10/B10,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <f aca="false">SUM(B5:B10)</f>
+        <v>16560000</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <f aca="false">SUM(C5:C10)</f>
+        <v>869400</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <f aca="false">SUM(D5:D10)</f>
+        <v>186300</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <f aca="false">SUM(E5:E10)</f>
+        <v>207000</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <f aca="false">SUM(F5:F10)</f>
+        <v>393300</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <f aca="false">SUM(G5:G10)</f>
+        <v>117990</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <f aca="false">IFERROR(F11/B11,0)</f>
+        <v>0.02375</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="20" t="n">
+        <f aca="false">F11-月度测算!N13</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:E13"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>